<commit_message>
UI: Add modern centered modal dialog with red and gray pill buttons for delete confirmation
</commit_message>
<xml_diff>
--- a/campus_ledger.xlsx
+++ b/campus_ledger.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Entry_ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -492,7 +502,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Admissions</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>DOC-1000</t>
         </is>
       </c>
     </row>
@@ -530,7 +550,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Examination Branch</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>DOC-1001</t>
         </is>
       </c>
     </row>
@@ -550,10 +580,8 @@
           <t>PADARTHI VAMSIKRISHNA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>113119071</t>
-        </is>
+      <c r="D4" t="n">
+        <v>113119071</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -570,7 +598,341 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Examination Branch</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>DOC-1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:53:24</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Study &amp; Conduct Certificate</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PADARTHI VAMSI KRISHNA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5831</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>General Administration</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>DOC-1003</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-18 17:08:32</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Study &amp; Conduct Certificate</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PADARTHI VAMSI KRISHNA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5831</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>General Administration</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>DOC-1004</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-18 17:08:32</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pass Certificate cum Memorandum of Marks</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PADARTHI VAMSIKRISHNA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1108210283</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MPC (Mathematics, Physics, Chemistry)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>686/1000 (B GRADE)</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Examination Branch</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>DOC-1005</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-18 17:08:32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fee Receipt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rahul Kumar</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TEST2026-00451</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Computer Science &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>39750</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Accounts &amp; Finance</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>DOC-1006</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-18 18:47:12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Study &amp; Conduct Certificate</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PADARTHI VAMSI KRISHNA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>5831</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>General Administration</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>DOC-1789737432353</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-18 18:52:09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pass Certificate cum Memorandum of Marks</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PADARTHI VAMSIKRISHNA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1108210283</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mathematics, Physics, Chemistry (MPC)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>686/1000 (B Grade)</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Examination Branch</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>DOC-1789737729574</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-18 18:55:34</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fee Receipt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rahul Kumar</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TEST-2026-00125</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Computer Science &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>39750</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Accounts &amp; Finance</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DOC-1789737934935</t>
         </is>
       </c>
     </row>

</xml_diff>